<commit_message>
Rekenkern: tracés opsplitsen op eigenschappen, aftakkingen, boringen en mantelbuizen
Knipt niet meer op elke zonegrens. Elk sub-tracé krijgt de zwaarste zone en
haaks/evenwijdig als kenmerk; delen buiten de zones vallen af. Stukjes < 5 m
gaan op in hun tak (niet naast een boring of mantelbuis), elke boring is apart,
alle mantelbuizen samen zijn een sub-tracé, huisaansluitingen horen bij hun tak.
De app toetst nu per sub-tracé. Testgevallen voor scenario 1-6 in test_opsplitsen.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KrMScywchu3hdzyhxi1uDm
</commit_message>
<xml_diff>
--- a/regeltemplate_v4_AGV.xlsx
+++ b/regeltemplate_v4_AGV.xlsx
@@ -493,7 +493,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -550,7 +549,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -565,7 +563,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -587,7 +584,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -721,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -828,7 +824,27 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Tracédelen korter dan dit worden samengevoegd met het buurdeel (ruis bij zonegrenzen).</t>
+          <t>Lijnen waarvan de uiteinden binnen deze afstand liggen, zitten aan elkaar vast (aftakking of doorlopende leiding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KORT_STUK_M</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>meter</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Stukjes korter dan dit, zonder andere zone, gaan op in de tak waar ze aan vastzitten (niet naast een boring of mantelbuis).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Opsplitsen: putsymbolen en losse kolkaansluitingen geven geen extra sub-tracés
Kleine lijntjes (<= KRUIMEL_M) zijn geen knip of aftakking. Aansluitingen uit
meerdere stukjes gaan samen; een losse aansluiting hoort bij het dichtstbijzijnde
sub-tracé binnen HA_ZOEKAFSTAND_M. Omval (11.0058) nieuw: 11 -> 3 sub-tracés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KrMScywchu3hdzyhxi1uDm
</commit_message>
<xml_diff>
--- a/regeltemplate_v4_AGV.xlsx
+++ b/regeltemplate_v4_AGV.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -845,6 +845,46 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>Stukjes korter dan dit, zonder andere zone, gaan op in de tak waar ze aan vastzitten (niet naast een boring of mantelbuis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KRUIMEL_M</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>meter</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Lijntjes die niet groter zijn dan dit (bijv. een putsymbool) zijn geen knip of aftakking en gaan op in de leiding ernaast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HA_ZOEKAFSTAND_M</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>meter</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Een huis- of kolkaansluiting die nergens aan vastzit, hoort bij het dichtstbijzijnde sub-tracé binnen deze afstand.</t>
         </is>
       </c>
     </row>

</xml_diff>